<commit_message>
Apostolados mensuales ya con fecha definida (jul-dic)
29 jul, 19 ago, 23 sep, 14 oct (mie), 14 nov (sab) y 9 dic (mie).
Antes aparecian al final de cada mes como "fecha por definir";
ahora quedan en su dia, con la nota "Lugar por definir".

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -803,8 +803,14 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
+      <c r="B10" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -818,7 +824,7 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Lugar y fecha exacta por definir</t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
@@ -1021,16 +1027,20 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F16" s="2" t="n"/>
-      <c r="G16" s="3" t="n"/>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="2" t="n"/>
@@ -1041,24 +1051,26 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
+      <c r="B17" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F17" s="2" t="n"/>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Lugar y fecha exacta por definir</t>
-        </is>
-      </c>
+      <c r="G17" s="3" t="n"/>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="2" t="n"/>
@@ -1305,8 +1317,14 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
+      <c r="B25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -1320,7 +1338,7 @@
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Lugar y fecha exacta por definir</t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H25" s="2" t="n"/>
@@ -1495,8 +1513,14 @@
           <t>Octubre</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
+      <c r="B31" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -1510,7 +1534,7 @@
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Lugar y fecha exacta por definir</t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H31" s="2" t="n"/>
@@ -1741,8 +1765,14 @@
           <t>Noviembre</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
+      <c r="B39" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Sáb</t>
+        </is>
+      </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -1756,7 +1786,7 @@
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Lugar y fecha exacta por definir</t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H39" s="2" t="n"/>
@@ -1937,8 +1967,14 @@
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
+      <c r="B45" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -1952,7 +1988,7 @@
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Lugar y fecha exacta por definir</t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H45" s="2" t="n"/>

</xml_diff>

<commit_message>
Septiembre: quita Misa de Niños (6 sep) y renombra la misa del 27 a «Misa Mensual - Misa de niños»
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1220,33 +1220,25 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Misa de Niños</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>Junta de Consejo</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="3" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="2" t="n"/>
@@ -1258,21 +1250,21 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Kermés de la Parroquia La Resurrección</t>
         </is>
       </c>
       <c r="F23" s="2" t="n"/>
@@ -1288,25 +1280,29 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Kermés de la Parroquia La Resurrección</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F24" s="2" t="n"/>
-      <c r="G24" s="3" t="n"/>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="2" t="n"/>
@@ -1327,20 +1323,16 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F25" s="2" t="n"/>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G25" s="3" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="2" t="n"/>
@@ -1352,25 +1344,33 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="3" t="n"/>
+          <t>Misa Mensual - Misa de niños</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="2" t="n"/>
@@ -1382,33 +1382,25 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="3" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="2" t="n"/>
@@ -1416,25 +1408,25 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Septiembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F28" s="2" t="n"/>
@@ -1450,25 +1442,29 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
         </is>
       </c>
       <c r="F29" s="2" t="n"/>
-      <c r="G29" s="3" t="n"/>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="2" t="n"/>
@@ -1480,27 +1476,27 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H30" s="2" t="n"/>
@@ -1514,7 +1510,7 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
@@ -1523,20 +1519,16 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F31" s="2" t="n"/>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G31" s="3" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="2" t="n"/>
@@ -1548,21 +1540,21 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Actividad económica grande (Conferencias)</t>
         </is>
       </c>
       <c r="F32" s="2" t="n"/>
@@ -1578,25 +1570,33 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Actividad económica grande (Conferencias)</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="3" t="n"/>
+          <t>Misa mensual</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="2" t="n"/>
@@ -1608,33 +1608,25 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="3" t="n"/>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="2" t="n"/>
@@ -1646,21 +1638,21 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Inicio de invitaciones para el Retiro de Compromiso 1</t>
         </is>
       </c>
       <c r="F35" s="2" t="n"/>
@@ -1672,25 +1664,25 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Inicio de invitaciones para el Retiro de Compromiso 1</t>
+          <t>Inicio de la Mega Rifa</t>
         </is>
       </c>
       <c r="F36" s="2" t="n"/>
@@ -1706,21 +1698,21 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Inicio de la Mega Rifa</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F37" s="2" t="n"/>
@@ -1736,25 +1728,29 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F38" s="2" t="n"/>
-      <c r="G38" s="3" t="n"/>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="2" t="n"/>
@@ -1766,27 +1762,31 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="n"/>
+          <t>Misa mensual y convivencia con KIDS</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Lugar por definir</t>
+          <t>(O apostolado con KIDS, por definir.)</t>
         </is>
       </c>
       <c r="H39" s="2" t="n"/>
@@ -1800,33 +1800,25 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual y convivencia con KIDS</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>(O apostolado con KIDS, por definir.)</t>
-        </is>
-      </c>
+          <t>Junta de Consejo</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="3" t="n"/>
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="2" t="n"/>
@@ -1838,21 +1830,21 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F41" s="2" t="n"/>
@@ -1864,25 +1856,25 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F42" s="2" t="n"/>
@@ -1897,27 +1889,37 @@
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
-        <v>2</v>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>4 – 6</t>
+        </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Vie a Dom</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Retiro de Compromiso</t>
         </is>
       </c>
       <c r="F43" s="2" t="n"/>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="2" t="n"/>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Retiro de compromiso INI#1 HMO</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="2" t="n"/>
     </row>
@@ -1927,37 +1929,31 @@
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>4 – 6</t>
-        </is>
+      <c r="B44" s="2" t="n">
+        <v>9</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Vie a Dom</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Retiro de Compromiso</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Retiro de compromiso INI#1 HMO</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="2" t="n"/>
     </row>
@@ -1968,29 +1964,25 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Mega Rifa</t>
         </is>
       </c>
       <c r="F45" s="2" t="n"/>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G45" s="3" t="n"/>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="2" t="n"/>
@@ -2002,21 +1994,21 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Vie</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Mega Rifa</t>
+          <t>Peregrinación</t>
         </is>
       </c>
       <c r="F46" s="2" t="n"/>
@@ -2032,11 +2024,11 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Vie</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2046,7 +2038,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Peregrinación</t>
+          <t>Día de la Virgen, misa y Posada KIDS</t>
         </is>
       </c>
       <c r="F47" s="2" t="n"/>
@@ -2062,11 +2054,11 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2076,11 +2068,15 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Día de la Virgen, misa y Posada KIDS</t>
+          <t>Posada durante la junta</t>
         </is>
       </c>
       <c r="F48" s="2" t="n"/>
-      <c r="G48" s="3" t="n"/>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Última junta del mes de diciembre.</t>
+        </is>
+      </c>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="2" t="n"/>
@@ -2092,29 +2088,25 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Posada durante la junta</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F49" s="2" t="n"/>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Última junta del mes de diciembre.</t>
-        </is>
-      </c>
+      <c r="G49" s="3" t="n"/>
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="2" t="n"/>
@@ -2126,21 +2118,21 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Jue</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Última Hora Santa del año</t>
         </is>
       </c>
       <c r="F50" s="2" t="n"/>
@@ -2148,36 +2140,6 @@
       <c r="H50" s="2" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="2" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Jue</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>Última Hora Santa del año</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="3" t="n"/>
-      <c r="J51" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H52"/>

</xml_diff>

<commit_message>
Junta de Consejo: agosto pasa del miércoles 19 al martes 18 y se agrega el miércoles 2 de septiembre
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1052,11 +1052,11 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1179,37 +1179,27 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>4 – 6</t>
-        </is>
+      <c r="B21" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Vie a Dom</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Retiro #3 de Chihuahua</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F21" s="2" t="n"/>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Nos unimos todos en oración</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="2" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="2" t="n"/>
     </row>
@@ -1219,27 +1209,37 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
-        <v>9</v>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>4 – 6</t>
+        </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Vie a Dom</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Retiro #3 de Chihuahua</t>
         </is>
       </c>
       <c r="F22" s="2" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="2" t="n"/>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Nos unimos todos en oración</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="2" t="n"/>
     </row>
@@ -1250,21 +1250,21 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Kermés de la Parroquia La Resurrección</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F23" s="2" t="n"/>
@@ -1280,29 +1280,25 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Kermés de la Parroquia La Resurrección</t>
         </is>
       </c>
       <c r="F24" s="2" t="n"/>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G24" s="3" t="n"/>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="2" t="n"/>
@@ -1323,16 +1319,20 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F25" s="2" t="n"/>
-      <c r="G25" s="3" t="n"/>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="2" t="n"/>
@@ -1344,33 +1344,25 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Misa Mensual - Misa de niños</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>Junta de Consejo</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="3" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="2" t="n"/>
@@ -1382,25 +1374,33 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="3" t="n"/>
+          <t>Misa Mensual - Misa de niños</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="2" t="n"/>
@@ -1408,25 +1408,25 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Septiembre</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F28" s="2" t="n"/>
@@ -1442,29 +1442,25 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F29" s="2" t="n"/>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
-        </is>
-      </c>
+      <c r="G29" s="3" t="n"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="2" t="n"/>
@@ -1476,27 +1472,27 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
         </is>
       </c>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Lugar por definir</t>
+          <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
         </is>
       </c>
       <c r="H30" s="2" t="n"/>
@@ -1510,7 +1506,7 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
@@ -1519,16 +1515,20 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F31" s="2" t="n"/>
-      <c r="G31" s="3" t="n"/>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="2" t="n"/>
@@ -1540,21 +1540,21 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Actividad económica grande (Conferencias)</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F32" s="2" t="n"/>
@@ -1570,33 +1570,25 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>Actividad económica grande (Conferencias)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="3" t="n"/>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="2" t="n"/>
@@ -1608,25 +1600,33 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="3" t="n"/>
+          <t>Misa mensual</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="2" t="n"/>
@@ -1638,21 +1638,21 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Inicio de invitaciones para el Retiro de Compromiso 1</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F35" s="2" t="n"/>
@@ -1664,25 +1664,25 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Inicio de la Mega Rifa</t>
+          <t>Inicio de invitaciones para el Retiro de Compromiso 1</t>
         </is>
       </c>
       <c r="F36" s="2" t="n"/>
@@ -1698,21 +1698,21 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Inicio de la Mega Rifa</t>
         </is>
       </c>
       <c r="F37" s="2" t="n"/>
@@ -1728,29 +1728,25 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F38" s="2" t="n"/>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G38" s="3" t="n"/>
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="2" t="n"/>
@@ -1762,31 +1758,27 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual y convivencia con KIDS</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
+          <t>Apostolado mensual</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n"/>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>(O apostolado con KIDS, por definir.)</t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H39" s="2" t="n"/>
@@ -1800,25 +1792,33 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="3" t="n"/>
+          <t>Misa mensual y convivencia con KIDS</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>(O apostolado con KIDS, por definir.)</t>
+        </is>
+      </c>
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="2" t="n"/>
@@ -1830,21 +1830,21 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F41" s="2" t="n"/>
@@ -1856,25 +1856,25 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F42" s="2" t="n"/>
@@ -1889,37 +1889,27 @@
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>4 – 6</t>
-        </is>
+      <c r="B43" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Vie a Dom</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Retiro de Compromiso</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F43" s="2" t="n"/>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Retiro de compromiso INI#1 HMO</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="2" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="2" t="n"/>
     </row>
@@ -1929,31 +1919,37 @@
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
-        <v>9</v>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>4 – 6</t>
+        </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Vie a Dom</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Retiro de Compromiso</t>
         </is>
       </c>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="n"/>
+          <t>Retiro de compromiso INI#1 HMO</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="2" t="n"/>
     </row>
@@ -1964,25 +1960,29 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Mega Rifa</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F45" s="2" t="n"/>
-      <c r="G45" s="3" t="n"/>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="2" t="n"/>
@@ -1994,21 +1994,21 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Vie</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Peregrinación</t>
+          <t>Mega Rifa</t>
         </is>
       </c>
       <c r="F46" s="2" t="n"/>
@@ -2024,11 +2024,11 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Vie</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Día de la Virgen, misa y Posada KIDS</t>
+          <t>Peregrinación</t>
         </is>
       </c>
       <c r="F47" s="2" t="n"/>
@@ -2054,11 +2054,11 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2068,15 +2068,11 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Posada durante la junta</t>
+          <t>Día de la Virgen, misa y Posada KIDS</t>
         </is>
       </c>
       <c r="F48" s="2" t="n"/>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Última junta del mes de diciembre.</t>
-        </is>
-      </c>
+      <c r="G48" s="3" t="n"/>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="2" t="n"/>
@@ -2088,25 +2084,29 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Posada durante la junta</t>
         </is>
       </c>
       <c r="F49" s="2" t="n"/>
-      <c r="G49" s="3" t="n"/>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Última junta del mes de diciembre.</t>
+        </is>
+      </c>
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="2" t="n"/>
@@ -2118,21 +2118,21 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Jue</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Última Hora Santa del año</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F50" s="2" t="n"/>
@@ -2140,6 +2140,36 @@
       <c r="H50" s="2" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Especial</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Última Hora Santa del año</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="3" t="n"/>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="3" t="n"/>
+      <c r="J51" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H52"/>

</xml_diff>

<commit_message>
Diciembre: la Posada pasa al miércoles 16 (ya no durante la junta del 14)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -2084,11 +2084,11 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2098,15 +2098,11 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Posada durante la junta</t>
+          <t>Posada</t>
         </is>
       </c>
       <c r="F49" s="2" t="n"/>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Última junta del mes de diciembre.</t>
-        </is>
-      </c>
+      <c r="G49" s="3" t="n"/>
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="2" t="n"/>

</xml_diff>

<commit_message>
Diciembre: se cancela la Mega Rifa del martes 8
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1994,21 +1994,21 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Vie</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Mega Rifa</t>
+          <t>Peregrinación</t>
         </is>
       </c>
       <c r="F46" s="2" t="n"/>
@@ -2024,11 +2024,11 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Vie</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Peregrinación</t>
+          <t>Día de la Virgen, misa y Posada KIDS</t>
         </is>
       </c>
       <c r="F47" s="2" t="n"/>
@@ -2054,11 +2054,11 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Día de la Virgen, misa y Posada KIDS</t>
+          <t>Posada</t>
         </is>
       </c>
       <c r="F48" s="2" t="n"/>
@@ -2093,12 +2093,12 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Posada</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F49" s="2" t="n"/>
@@ -2114,21 +2114,21 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Jue</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Última Hora Santa del año</t>
         </is>
       </c>
       <c r="F50" s="2" t="n"/>
@@ -2137,49 +2137,19 @@
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="2" t="n"/>
     </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Jue</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>Última Hora Santa del año</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="3" t="n"/>
-      <c r="J51" s="2" t="n"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:H52"/>
   <dataValidations count="4">
-    <dataValidation sqref="A2:A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="A2:A50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junta de Consejo,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Juntas de Consejo cada 2 semanas desde el 30 sep; agrega Lunada, Conferencias y Limpieza de rancho
- Junta de Consejo: 30 sep, 14 oct, 28 oct, 11 nov, 25 nov y 9 dic
  (se quitan 7 oct, 21 oct, 4 nov, 18 nov, 2 dic y 16 dic).
- Desde el calendario de Comunidad: Lunada en el Rancho (sáb 24 – dom 25 oct),
  Conferencias ÉL VIVE pasan del 24 oct al miércoles 25 nov y
  Limpieza de rancho el sábado 28 nov.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1438,11 +1438,11 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Septiembre</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
@@ -1566,11 +1566,11 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Actividad económica grande (Conferencias)</t>
+          <t>Conferencias ÉL VIVE</t>
         </is>
       </c>
       <c r="F33" s="2" t="n"/>
@@ -1724,11 +1724,11 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
@@ -1886,11 +1886,11 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
@@ -2137,19 +2137,85 @@
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="2" t="n"/>
     </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>24 – 25</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Sáb a Dom</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Especial</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Lunada en el Rancho</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="3" t="n"/>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="n"/>
+      <c r="J51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Sáb</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Especial</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Limpieza de rancho</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="3" t="n"/>
+      <c r="H52" s="2" t="n"/>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="2" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H52"/>
   <dataValidations count="4">
-    <dataValidation sqref="A2:A50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="A2:A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junta de Consejo,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Quita limpieza de rancho del 10 oct y Mega Rifa del 2 nov; iguala apostolados y misas con Comunidad
- Se eliminan: Primera limpieza de rancho (sáb 10 oct) e Inicio de la Mega Rifa (lun 2 nov).
- Apostolados como en Comunidad: el del 1 jul lleva hora 8:00 p.m. y se quita el del 14 oct.
- Misas como en Comunidad: la del domingo 27 sep pasa a llamarse «Misa Mensual».

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,11 @@
           <t>Apostolado mensual</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Hospital General del Estado (Blvd. Colosio y Quintero Arce)</t>
@@ -1388,7 +1392,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Misa Mensual - Misa de niños</t>
+          <t>Misa Mensual</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1472,29 +1476,25 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F30" s="2" t="n"/>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
-        </is>
-      </c>
+      <c r="G30" s="3" t="n"/>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="2" t="n"/>
@@ -1502,33 +1502,29 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Conferencias ÉL VIVE</t>
         </is>
       </c>
       <c r="F31" s="2" t="n"/>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G31" s="3" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="2" t="n"/>
@@ -1540,25 +1536,33 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="3" t="n"/>
+          <t>Misa mensual</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="2" t="n"/>
@@ -1566,25 +1570,25 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Conferencias ÉL VIVE</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F33" s="2" t="n"/>
@@ -1600,33 +1604,25 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>Inicio de invitaciones para el Retiro de Compromiso 1</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="3" t="n"/>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="2" t="n"/>
@@ -1638,21 +1634,21 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F35" s="2" t="n"/>
@@ -1664,29 +1660,33 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Inicio de invitaciones para el Retiro de Compromiso 1</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F36" s="2" t="n"/>
-      <c r="G36" s="3" t="n"/>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="2" t="n"/>
@@ -1698,25 +1698,33 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Inicio de la Mega Rifa</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="3" t="n"/>
+          <t>Misa mensual y convivencia con KIDS</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>(O apostolado con KIDS, por definir.)</t>
+        </is>
+      </c>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="2" t="n"/>
@@ -1724,11 +1732,11 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
@@ -1758,29 +1766,25 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F39" s="2" t="n"/>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G39" s="3" t="n"/>
       <c r="H39" s="2" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="2" t="n"/>
@@ -1792,33 +1796,25 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual y convivencia con KIDS</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>(O apostolado con KIDS, por definir.)</t>
-        </is>
-      </c>
+          <t>Junta de Consejo</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="3" t="n"/>
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="2" t="n"/>
@@ -1826,59 +1822,73 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n">
-        <v>11</v>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>4 – 6</t>
+        </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Vie a Dom</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Retiro de Compromiso</t>
         </is>
       </c>
       <c r="F41" s="2" t="n"/>
-      <c r="G41" s="3" t="n"/>
-      <c r="H41" s="2" t="n"/>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Retiro de compromiso INI#1 HMO</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="2" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F42" s="2" t="n"/>
-      <c r="G42" s="3" t="n"/>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H42" s="2" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="2" t="n"/>
@@ -1886,25 +1896,25 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Vie</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Peregrinación</t>
         </is>
       </c>
       <c r="F43" s="2" t="n"/>
@@ -1919,14 +1929,12 @@
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>4 – 6</t>
-        </is>
+      <c r="B44" s="2" t="n">
+        <v>12</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Vie a Dom</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1936,20 +1944,12 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Retiro de Compromiso</t>
+          <t>Día de la Virgen, misa y Posada KIDS</t>
         </is>
       </c>
       <c r="F44" s="2" t="n"/>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Retiro de compromiso INI#1 HMO</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
+      <c r="G44" s="3" t="n"/>
+      <c r="H44" s="2" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="2" t="n"/>
     </row>
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
@@ -1969,20 +1969,16 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
+          <t>Posada</t>
         </is>
       </c>
       <c r="F45" s="2" t="n"/>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+      <c r="G45" s="3" t="n"/>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="2" t="n"/>
@@ -1994,21 +1990,21 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Vie</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Peregrinación</t>
+          <t>Junta de Consejo</t>
         </is>
       </c>
       <c r="F46" s="2" t="n"/>
@@ -2024,11 +2020,11 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Jue</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2038,7 +2034,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Día de la Virgen, misa y Posada KIDS</t>
+          <t>Última Hora Santa del año</t>
         </is>
       </c>
       <c r="F47" s="2" t="n"/>
@@ -2050,15 +2046,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>16</v>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>24 – 25</t>
+        </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Sáb a Dom</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2068,37 +2066,41 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Posada</t>
+          <t>Lunada en el Rancho</t>
         </is>
       </c>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="3" t="n"/>
-      <c r="H48" s="2" t="n"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Junta de Consejo</t>
+          <t>Limpieza de rancho</t>
         </is>
       </c>
       <c r="F49" s="2" t="n"/>
@@ -2107,115 +2109,19 @@
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="2" t="n"/>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Jue</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>Última Hora Santa del año</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="n"/>
-      <c r="G50" s="3" t="n"/>
-      <c r="H50" s="2" t="n"/>
-      <c r="I50" s="3" t="n"/>
-      <c r="J50" s="2" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Octubre</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>24 – 25</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Sáb a Dom</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>Lunada en el Rancho</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I51" s="3" t="n"/>
-      <c r="J51" s="2" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Noviembre</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Sáb</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>Limpieza de rancho</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="3" t="n"/>
-      <c r="H52" s="2" t="n"/>
-      <c r="I52" s="3" t="n"/>
-      <c r="J52" s="2" t="n"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:H52"/>
   <dataValidations count="4">
-    <dataValidation sqref="A2:A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="A2:A49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junta de Consejo,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>